<commit_message>
V1.8.4-rc1: Implement RMCSA reading practice mode
</commit_message>
<xml_diff>
--- a/public/database/RMCSA/RMCSA/RMCSA.xlsx
+++ b/public/database/RMCSA/RMCSA/RMCSA.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -590,6 +590,32 @@
 [] New products are easy to distinguish from old ones.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that analyzing the main point of a passage requires you to look beyond the surface details and identify the author's central argument. This passage is excellent because it challenges a common misconception, which is exactly what PTE questions often test!&lt;/p&gt;
+&lt;p&gt;Let's break down the passage, the question, and each option to ensure you understand the logic behind the correct answer.&lt;/p&gt;
+&lt;h2&gt;✅ Analysis of the Correct Answer&lt;/h2&gt;
+&lt;p&gt;The correct option is: &lt;strong&gt;New products are not always based on new ideas.&lt;/strong&gt;&lt;/p&gt;
+&lt;h3&gt;Why this is correct:&lt;/h3&gt;
+&lt;p&gt;This option perfectly captures the writer's main point, which is a critique of the popular belief that all innovations are sudden acts of genius. The passage repeatedly argues that the source of new technology is often pre-existing or adapted.&lt;/p&gt;
+&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Passage Evidence:&lt;/strong&gt; The text states, "The fact is that innovations were often already 'out there' in the public domain in some form or another."&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Passage Evidence:&lt;/strong&gt; It continues, "They tend to evolve from notions that have been around for years but that had not, until that point, been suitably adapted."&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;The core message is that innovation is less about creating something entirely new (a "genius" idea) and more about &lt;strong&gt;adapting&lt;/strong&gt; or &lt;strong&gt;combining&lt;/strong&gt; existing, overlooked ideas. Therefore, the main point is that the ideas themselves are not always brand new.&lt;/p&gt;
+&lt;h2&gt;❌ Analysis of the Incorrect Answers&lt;/h2&gt;
+&lt;p&gt;Understanding why the other options are wrong is just as important as knowing the right answer. It helps you eliminate distractors!&lt;/p&gt;
+&lt;h3&gt;1. Many new products fail to interest consumers.&lt;/h3&gt;
+&lt;p&gt;&lt;strong&gt;Why it is incorrect:&lt;/strong&gt; The passage never discusses consumer interest, market failure, or consumer reception. The entire focus is on the &lt;em&gt;origin&lt;/em&gt; and &lt;em&gt;development&lt;/em&gt; of the idea, not its commercial success. This option introduces information that is completely irrelevant to the text.&lt;/p&gt;
+&lt;h3&gt;2. Creators of new products require a unique set of skills.&lt;/h3&gt;
+&lt;p&gt;&lt;strong&gt;Why it is incorrect:&lt;/strong&gt; This option misinterprets the passage's focus. While the passage mentions "vision and insight," it immediately refutes the idea that this requires a unique, singular genius. Instead, it suggests that the required skill is often the ability to &lt;strong&gt;adapt&lt;/strong&gt; or &lt;strong&gt;combine&lt;/strong&gt; existing concepts, rather than generating a wholly unique idea from scratch. The passage is about the &lt;em&gt;idea's source&lt;/em&gt;, not the &lt;em&gt;creator's skill set&lt;/em&gt;.&lt;/p&gt;
+&lt;h3&gt;3. New products are easy to distinguish from old ones.&lt;/h3&gt;
+&lt;p&gt;&lt;strong&gt;Why it is incorrect:&lt;/strong&gt; This option directly contradicts the passage's description of the innovation process. The passage describes the "long nose" approach, where concepts come into the world &lt;strong&gt;slowly, gradually revealing all they have to offer&lt;/strong&gt;. This suggests a subtle, gradual evolution, making them difficult to distinguish from their older, foundational forms, rather than being instantly obvious or radically different.&lt;/p&gt;
+&lt;h2&gt;💡 Summary Tip for PTE Reading&lt;/h2&gt;
+&lt;p&gt;When faced with a "Main Point" question, always ask yourself: &lt;strong&gt;"What is the author trying to convince me of?"&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;In this case, the author is trying to convince you that the myth of the "genius inventor" is wrong, and that innovation is a process of &lt;strong&gt;adaptation&lt;/strong&gt;. This realization leads directly to the correct answer!&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">

</xml_diff>

<commit_message>
V1.8.8 - Implement HCS & RMCSA, Optimize HIW & SMW, and Unify UI Elements
</commit_message>
<xml_diff>
--- a/public/database/RMCSA/RMCSA/RMCSA.xlsx
+++ b/public/database/RMCSA/RMCSA/RMCSA.xlsx
@@ -488,7 +488,7 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that analyzing reading passages requires you to be extremely precise—you must only use the information given in the text. Let's break down this passage and question together. You did a great job identifying the correct answer, and now we will solidify your understanding of why the others are incorrect!&lt;/p&gt;
-&lt;h2&gt;✅ Analysis of the Correct Answer&lt;/h2&gt;
+&lt;h3&gt;✅ Analysis of the Correct Answer&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;Cathedral staff were reluctant to act too quickly.&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Why this is correct:&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
@@ -496,7 +496,7 @@
     &lt;li&gt;When the clergy was asked to synchronize, they "discussed the request but decided that this was an idea that needed to prove its worth before being adopted."&lt;/li&gt;
 &lt;/ul&gt;
 &lt;p&gt;This decision to wait and require proof before making a change perfectly aligns with the idea of being &lt;strong&gt;"reluctant to act too quickly."&lt;/strong&gt; The passage attributes the delay not to mechanical difficulty, but to a cautious, deliberative decision by the staff/clergy.&lt;/p&gt;
-&lt;h2&gt;❌ Analysis of the Incorrect Answers&lt;/h2&gt;
+&lt;h3&gt;❌ Analysis of the Incorrect Answers&lt;/h3&gt;
 &lt;p&gt;It is crucial in PTE reading to avoid making assumptions about the text. Let's look at why the other options fail:&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;1. Oxford likes to be different from other places.&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
@@ -510,7 +510,7 @@
 &lt;ul&gt;
     &lt;li&gt;&lt;strong&gt;Why it is wrong:&lt;/strong&gt; This option introduces information that is not mentioned in the passage. The passage focuses entirely on the &lt;strong&gt;decision&lt;/strong&gt; (the clergy's choice to delay the change), not the &lt;strong&gt;physical difficulty&lt;/strong&gt; of the clock mechanism. We cannot assume the clock was hard to change just because the clergy chose not to change it.&lt;/li&gt;
 &lt;/ul&gt;
-&lt;h2&gt;💡 Key Takeaway for PTE Success&lt;/h2&gt;
+&lt;h3&gt;💡 Key Takeaway for PTE Success&lt;/h3&gt;
 &lt;p&gt;When tackling these questions, remember this rule: &lt;strong&gt;The passage is your only source of truth.&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;If an option requires you to guess the motivation (like "Oxford likes to be different") or introduces external facts (like "it was mechanically difficult"), it is likely incorrect, even if it seems plausible. Always look for the direct cause-and-effect relationship described in the text!&lt;/p&gt;</t>
         </is>
@@ -540,7 +540,7 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that mastering the "Main Purpose" question is all about reading between the lines and identifying the author's core message. Don't get distracted by the details; focus on the big picture! Let's break down this passage together.&lt;/p&gt;
-&lt;h2&gt;🎯 Analysis of the Correct Answer&lt;/h2&gt;
+&lt;h3&gt;🎯 Analysis of the Correct Answer&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;to highlight the potential benefits of geothermal power for Britain&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Why this is correct:&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
@@ -548,7 +548,7 @@
     &lt;li&gt;&lt;strong&gt;The Core Message:&lt;/strong&gt; While the passage does mention difficulties (extraction is "difficult and expensive"), these challenges are presented as obstacles *against* a massive, desirable potential. The writer's primary goal is to make you realize how much energy Britain *could* have, making the potential benefit the central theme.&lt;/li&gt;
     &lt;li&gt;&lt;strong&gt;Key Evidence:&lt;/strong&gt; The phrases "Huge reserves," "provide power for millions of homes," and "keep regenerating indefinitely" all point toward the immense, positive potential.&lt;/li&gt;
 &lt;/ul&gt;
-&lt;h2&gt;❌ Analysis of the Incorrect Answers&lt;/h2&gt;
+&lt;h3&gt;❌ Analysis of the Incorrect Answers&lt;/h3&gt;
 &lt;p&gt;Understanding why the other options are wrong is just as important as knowing the right answer. It helps you avoid common traps!&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;1. to show how common the use of geothermal power is in Britain&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
@@ -562,7 +562,7 @@
 &lt;ul&gt;
     &lt;li&gt;&lt;strong&gt;Why it is wrong:&lt;/strong&gt; The passage is descriptive, but it is not a detailed scientific guide. It mentions the need for "Thousands of bore holes," which is a procedural detail, but it does not explain the complex scientific process of heat conversion or energy production in a detailed, step-by-step manner.&lt;/li&gt;
 &lt;/ul&gt;
-&lt;h2&gt;💡 PTE Strategy Takeaway&lt;/h2&gt;
+&lt;h3&gt;💡 PTE Strategy Takeaway&lt;/h3&gt;
 &lt;p&gt;When tackling "Main Purpose" questions, always ask yourself: &lt;strong&gt;"What is the single most important idea the writer wants me to walk away with?"&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;In this case, the writer wants you to be impressed by the sheer amount of untapped energy—the &lt;strong&gt;potential benefit&lt;/strong&gt;—even if the current reality is challenging.&lt;/p&gt;
 &lt;p&gt;Keep practicing, and remember to look for the overarching theme, not just the facts!&lt;/p&gt;</t>
@@ -594,7 +594,7 @@
         <is>
           <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that analyzing the main point of a passage requires you to look beyond the surface details and identify the author's central argument. This passage is excellent because it challenges a common misconception, which is exactly what PTE questions often test!&lt;/p&gt;
 &lt;p&gt;Let's break down the passage, the question, and each option to ensure you understand the logic behind the correct answer.&lt;/p&gt;
-&lt;h2&gt;✅ Analysis of the Correct Answer&lt;/h2&gt;
+&lt;h3&gt;✅ Analysis of the Correct Answer&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;New products are not always based on new ideas.&lt;/strong&gt;&lt;/p&gt;
 &lt;h3&gt;Why this is correct:&lt;/h3&gt;
 &lt;p&gt;This option perfectly captures the writer's main point, which is a critique of the popular belief that all innovations are sudden acts of genius. The passage repeatedly argues that the source of new technology is often pre-existing or adapted.&lt;/p&gt;
@@ -603,7 +603,7 @@
     &lt;li&gt;&lt;strong&gt;Passage Evidence:&lt;/strong&gt; It continues, "They tend to evolve from notions that have been around for years but that had not, until that point, been suitably adapted."&lt;/li&gt;
 &lt;/ul&gt;
 &lt;p&gt;The core message is that innovation is less about creating something entirely new (a "genius" idea) and more about &lt;strong&gt;adapting&lt;/strong&gt; or &lt;strong&gt;combining&lt;/strong&gt; existing, overlooked ideas. Therefore, the main point is that the ideas themselves are not always brand new.&lt;/p&gt;
-&lt;h2&gt;❌ Analysis of the Incorrect Answers&lt;/h2&gt;
+&lt;h3&gt;❌ Analysis of the Incorrect Answers&lt;/h3&gt;
 &lt;p&gt;Understanding why the other options are wrong is just as important as knowing the right answer. It helps you eliminate distractors!&lt;/p&gt;
 &lt;h3&gt;1. Many new products fail to interest consumers.&lt;/h3&gt;
 &lt;p&gt;&lt;strong&gt;Why it is incorrect:&lt;/strong&gt; The passage never discusses consumer interest, market failure, or consumer reception. The entire focus is on the &lt;em&gt;origin&lt;/em&gt; and &lt;em&gt;development&lt;/em&gt; of the idea, not its commercial success. This option introduces information that is completely irrelevant to the text.&lt;/p&gt;
@@ -611,7 +611,7 @@
 &lt;p&gt;&lt;strong&gt;Why it is incorrect:&lt;/strong&gt; This option misinterprets the passage's focus. While the passage mentions "vision and insight," it immediately refutes the idea that this requires a unique, singular genius. Instead, it suggests that the required skill is often the ability to &lt;strong&gt;adapt&lt;/strong&gt; or &lt;strong&gt;combine&lt;/strong&gt; existing concepts, rather than generating a wholly unique idea from scratch. The passage is about the &lt;em&gt;idea's source&lt;/em&gt;, not the &lt;em&gt;creator's skill set&lt;/em&gt;.&lt;/p&gt;
 &lt;h3&gt;3. New products are easy to distinguish from old ones.&lt;/h3&gt;
 &lt;p&gt;&lt;strong&gt;Why it is incorrect:&lt;/strong&gt; This option directly contradicts the passage's description of the innovation process. The passage describes the "long nose" approach, where concepts come into the world &lt;strong&gt;slowly, gradually revealing all they have to offer&lt;/strong&gt;. This suggests a subtle, gradual evolution, making them difficult to distinguish from their older, foundational forms, rather than being instantly obvious or radically different.&lt;/p&gt;
-&lt;h2&gt;💡 Summary Tip for PTE Reading&lt;/h2&gt;
+&lt;h3&gt;💡 Summary Tip for PTE Reading&lt;/h3&gt;
 &lt;p&gt;When faced with a "Main Point" question, always ask yourself: &lt;strong&gt;"What is the author trying to convince me of?"&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;In this case, the author is trying to convince you that the myth of the "genius inventor" is wrong, and that innovation is a process of &lt;strong&gt;adaptation&lt;/strong&gt;. This realization leads directly to the correct answer!&lt;/p&gt;</t>
         </is>
@@ -639,6 +639,33 @@
 [] Dirty submarines are endangering the well-being of the sea snails that attach themselves.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;As an expert PTE Academic tutor, I will provide a detailed, option-level explanation to help you understand how to select the correct answer based on the passage's evidence.&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;✅ Correct Answer Explanation&lt;/strong&gt;&lt;/h3&gt;
+&lt;p&gt;The correct option is: &lt;strong&gt;Sea snails are being carried by submarines to places where they harm other species.&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Support:&lt;/strong&gt; This option accurately summarizes the core problem described in the passage. The text states that the limpets "latch on to the submarines... potentially spreading disease in pristine ecosystems." This directly supports the idea that the snails are being transported (carried by submarines) to new locations where they pose a threat (harm other species/ecosystems).&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;❌ Incorrect Options Analysis&lt;/strong&gt;&lt;/h3&gt;
+&lt;ol&gt;
+    &lt;li&gt;&lt;strong&gt;Research into sea snails has been harming the animals themselves.&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;&lt;strong&gt;Reasoning:&lt;/strong&gt; This option is &lt;strong&gt;not supported&lt;/strong&gt; by the passage. The passage describes the limpets as the source of the threat (they are infected and spread disease), not that the research itself is harming them.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Sea snails are spreading diseases to the research scientists on submarines.&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;&lt;strong&gt;Reasoning:&lt;/strong&gt; This option is &lt;strong&gt;incorrectly focused&lt;/strong&gt;. The passage specifies that the threat is to the &lt;em&gt;ecosystem&lt;/em&gt; ("poses a threat to the ecosystem"), not to the human scientists operating the submarines.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Dirty submarines are endangering the well-being of the sea snails that attach themselves.&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;&lt;strong&gt;Reasoning:&lt;/strong&gt; This option changes the meaning and misidentifies the problem. The passage states that the limpets are the danger because they are infected and spread disease; the problem is not that the submarines are endangering the limpets.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ol&gt;
+&lt;p&gt;&lt;strong&gt;💡 PTE Strategy Tip:&lt;/strong&gt; When answering comprehension questions, always look for the option that captures the main idea or the primary conflict presented in the text. In this case, the conflict is the *transportation* of the *disease* (the problem) via the *submarines* (the mechanism).&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -662,6 +689,11 @@
 [] the use of state-of-the-art cameras</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; teachers who have practical experience in a creative field&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What does the Graphic Design degree offer students?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The Graphic Design degree provides students with a nurturing environment for learning, developing aesthetic appreciation and design skills with an emphasis on media and marketing.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;experience working on new magazines&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;the opportunity to apply for funds to help with their study&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;the use of state-of-the-art cameras&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -684,6 +716,11 @@
 [x] they assist in driving public issues.</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; they assist in driving public issues.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author considers statistics to be important because&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;While it may be the issues behind the statistics, rather than the statistics as such that command the public&amp;#x27;s attention, it must be recognised that it is the figures that inform these issues.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;they are recorded by official organisations.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;the general public have an interest in them.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;they are affected by plans and policies.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -706,6 +743,11 @@
 [] Human action has upset the balance of the natural environment.</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The number of species is constantly changing.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Why is it difficult to establish the number of species globally?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;This is probably due to the fact that new species are continually appearing, while at the same time existing species evolve and some become extinct.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;There are too many species to count them all.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Currently, more species are appearing than are becoming extinct.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Human action has upset the balance of the natural environment.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -729,6 +771,11 @@
 [] To perfect techniques of historical research.</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To apply Roman law to their own society.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What was the ultimate aim of legal scholarship?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;For example, they studied the records of cases that went to court, official letters that had survived, and so on to get a fuller picture of how people really lived and went about their business.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To purify the ancient legal system.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To promote humanism in general.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To perfect techniques of historical research.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -753,6 +800,11 @@
 [] Because other species have more complex eyes.</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Because evidence of its ancestors is almost impossible to find.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Why are researchers forced to look outside a specific species for clues to gradual development?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In the same way, it shouldn&amp;#x27;t be hard to believe that a complex eye could be formed by natural selection if it can be shown that there were numerous stages from a simple and imperfect eye to a complex and perfect one, with each development being useful to its &lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Because the eye is so complex and perfect already.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Because the eye cannot change without losing its usefulness.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Because other species have more complex eyes.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -775,6 +827,11 @@
 [x] Jupiter’s development as compared to the Sun</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Jupiter’s development as compared to the Sun&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is mainly talked about in this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;However, unlike the Sun, the unavailability of sufficient mass required to create the temperature which can initiate fusion reaction, Jupiter relatively got cooler over a period of time.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;comparison of Jupiter’s temperature with other planets&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;size of Jupiter compared to other planets&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Jupiter’s development as compared to Earth over a period&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -797,6 +854,11 @@
 [] The artist’s inspiration came from the observation towards animals.</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The artist’s inspiration came from his reflection.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What can be inferred from this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Some of his greatest pictures were inspired by Byron, and he had a Byronic power of self-identification with the forces of the sublime - in particular ‘the roaring of lions and the destructive sword’.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The artist’s inspiration came from the change of his age.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The artist had strong emotion.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The artist’s inspiration came from the observation towards animals.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -819,6 +881,11 @@
 [x] drought</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; drought&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What does this passage suggest climate change will bring to Australia?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Per capita, Australia is one of the world&amp;#x27;s largest producers of carbon dioxide and other gases that many scientists believe are helping to warm the Earth&amp;#x27;s atmosphere, causing climate upset.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;gas emissions&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;environmental activists&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;carbon dioxide&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -843,6 +910,11 @@
 [] the poor quality of English expression in assignments</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; students copying others’ work&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What problem does the way a paper should be submitted address?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In your assignment list, to the right of the assignment that you must submit, you will see an icon of a document beneath the submit column.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;assignments being misplaced by university staff&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;overcrowding in classrooms at peak times&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;the poor quality of English expression in assignments&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -865,6 +937,11 @@
 [] Art is directed in a way that it deliberately appeals to the emotions of people.</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Art is a difficult and complex form to explain.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the main idea of the passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;It encompasses a diverse range of human activities, creations and ways of expression, including music, literature, film, sculpture and paintings.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Wikipedia defines art under aesthetics, which is a branch of philosophy.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Music, literature, film and sculpture do not define art.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Art is directed in a way that it deliberately appeals to the emotions of people.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -887,6 +964,11 @@
 [] To bring some humor into his text.</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To illustrate his view about the use of language.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the main reason for the writer mentioning Rowley?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Those who heard his words commented on his wisdom.This raises all sorts of questions about language and how we perceive the world, questions that range from the philosophical to the politically correct (PC) use of language and the question of causing offense —&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Because he is a farm laborer.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To support the idea that we should be politically correct when talking about animals.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To bring some humor into his text.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -909,6 +991,11 @@
 [] Sales of e-books are likely to overtake sales of traditional books.</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; E-publishing has created new possibilities for writers.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following statements is true according to the text?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Many e-books arepublished by writers who do not have a readership through mainstream publishers, and this allowsthem to deal with material that mainstream publishers would consider too controversial or otherwiseunmarketable.The market is very much driven by th&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Publishing companies have been unable to adapt to the new market.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;E-books will radically alter our reading habits.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sales of e-books are likely to overtake sales of traditional books.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -931,6 +1018,11 @@
 [] transplant scholarly techniques</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; change the focus of a field of study&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author&amp;#x27;s main purpose is to __ from one field of study to another&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Black people were most influenced by those Euro-American tales whose functional meaning and aesthetic appeal had the greatest similarity to the tales with deep roots in their ancestral homeland.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;create a new field of study&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;discredit an existing field of study&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;transplant scholarly techniques&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -953,6 +1045,11 @@
 [x] Focusing on those whose crimes have involved damage to persons or property</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Focusing on those whose crimes have involved damage to persons or property&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The passage suggests that scholars in criminal justice could be criticized for which of the following?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Even as the number of females processed through juvenile courts climbs steadily, an implicit consensus remains among scholars in criminal justice that male adolescents define the delinquency problem in the United States.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Underestimating the seriousness of juvenile crime&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Rationalizing the distinction made between juveniles and adults in the legal system&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Concerning themselves too little with the prevention of juvenile delinquency&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -975,6 +1072,11 @@
 [] humidity of an area on a cat’s</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; level of a hormone on a field mouse’s readiness for mating&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;All of the following could be considered examples of exogenous influences on an organism EXCEPT the influence of the __ .&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Although she could not posit an unequivocal causal relationship between behavior and environmental change, Brown concluded that a change in tide schedule is one of several possible exogenous influences (those outside the organism) on the oysters&amp;#x27; rhythms.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;temperature of a region on a bear’s hibernation&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;salt level of a river on a fish’s migration&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;humidity of an area on a cat’s&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -997,6 +1099,11 @@
 [x] compare and contrast two novels</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; compare and contrast two novels&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The primary purpose of the passage is to __&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Many readers are convinced that the compelling mysteries of each plot conceal elaborate structures of allusion and fierce, though shadowy, moral ambitions that seem to indicate metaphysical intentions, though efforts by critics to articulate these intentions h&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;defend a controversial interpretation of two novels&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;explain the source of widely recognized responses to two novels&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;delineate broad differences between two novels&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1019,6 +1126,11 @@
 [] Viruses for use by molecular biologists</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Microorganisms resistant to drugs&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, the exchange of plasmids between different bacteria can results in which of the following?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The drug resistance is chiefly conferred by tiny circlets of genes, called plasmids, that can be exchanged between different strains and even different species of bacteria.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Therapeutically useful circlets of genes&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Anti-infective drugs like penicillin&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Viruses for use by molecular biologists&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1041,6 +1153,11 @@
 [] The War of Independence provoked strong criticisms by many Americans of the institution of slavery, but produced little substantive action against it.</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The War of Independence exposed to many Americans the contradiction of slavery in a country seeking its freedom and resulted in efforts to resolve that contradiction.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following best states the central idea of the passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;&amp;quot;It always appeared a most iniquitous scheme to me,&amp;quot;Abigail Adams wrote her husband in 1774, &amp;quot;to fight ourselves for what we are daily robbing and plundering from those who have as good a right to freedom as we have.&amp;quot;Many Americans besides Abigail Adams were s&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The War of Independence produced among many Black Americans a heightened consciousness of the inequities in American society.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The War of Independence strengthened the bonds of slavery of many Black Americans while intensifying their desire to be free.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The War of Independence provoked strong criticisms by many Americans of the institution of slavery, but produced little substantive action against it.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1063,6 +1180,11 @@
 [x] putting various meaningful elements together in one word</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; putting various meaningful elements together in one word&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, some abstract universal ideas can be expressed in Nahuatl by __&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;By the combination of radicals or semantic elements, single compound words can express complex conceptual relations, often of an abstract universal character.The tlamatinime (&amp;#x27;those who know&amp;#x27;) were able to use this rich stock of abstract terms to express the n&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;taking away from a word any reference to particular instances&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;removing a word from its associations with other words&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;giving a word a new and opposite meaning&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1085,6 +1207,11 @@
 [] Water becoming unfit to drink through the release of pollutants into it from a manufacturing plant</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The trapping of water in a sealed underground rock cavern through the action of an earthquake&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;It can be inferred that which of the following is most likely to be the subject of study by a geohydrologist?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The hydrologic cycle, a major topic in this science, is the complete cycle of phenomena through which water passes, beginning as atmospheric water vapor, passing into liquid and solid form as precipitation, thence along and into the ground surface, and finally&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Soft, porous rock being worn away by a waterfall&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Water depositing minerals on the banks of a gorge through which the water runs&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Water becoming unfit to drink through the release of pollutants into it from a manufacturing plant&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1107,6 +1234,11 @@
 [x] Difficulties surrounding laboratory production of specimens for study</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Difficulties surrounding laboratory production of specimens for study&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;It can be inferred from the passage that which of the following has been a factor influencing the extent to which research on mycorrhizal fungi has progressed?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Despite these difficulties, there has been important new work that suggests that this symbiotic association can be harnessed to achieve more economical use of costly superphosphate fertilizer and to permit better exploitation of cheaper, less soluble rock phos&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Lack of funding for such research&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Lack of immediate application of such research&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Lack of a method for identifying mycorrhizal fungi&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1129,6 +1261,11 @@
 [] predict an ethical crisis for</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; discuss the current state of technology in the field of biomaterials&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author&amp;#x27;s primary purpose is to __&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Although recent research has allowed us to stabilize the tissue-biomaterial interface by controlling either the chemical reactions or the microstructure of the biomaterial, our fundamental understanding of how implant devices adhere to tissues remains woefully&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;answer a theoretical question in the field of biomaterials&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;resolve a research dispute in the field of biomaterial&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;predict an ethical crisis for&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1151,6 +1288,11 @@
 [] Regarded as unimportant the development of fervent emotionalism in a portion of Afro-American poetry.</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Ignored at least some of the historical roots of Afro-American poetry.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;It can be inferred from the passage that, before Wagner, most students of Afro-American poetry did which of the following?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;But before Wagner a secular outlook that analyzed Black poetry solely within the context of political and social protest was dominant in the field.It is Wagner who first demonstrated the essential fusion of racial and religious feeling in Afro-American poetry.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Contributed appreciably to the transfer of political protest from Afro-American poetry to direct political action.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Analyzed fully the aspects of social protest to be found in such traditional forms of Afro-American poetry as the Black spiritual.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Regarded as unimportant the development of fervent emotionalism in a portion of Afro-American poetry.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1173,6 +1315,11 @@
 [x] In spaces between pieces of sediment</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; In spaces between pieces of sediment&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this passage , where is groundwater usually found?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Ordinary meteoric water is water that has soaked into the ground from the surface, from precipitation (rain and snow) and from lakes and streams.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Inside pieces of sand and gravel&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;On top of beds of rock&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;In fast rivers that are flowing beneath the soil&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1195,6 +1342,11 @@
 [x] To increase the society’s prosperity</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To increase the society’s prosperity&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According tothis passage, why did some societies develop and repeat ceremonial actions?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Having little understanding of natural causes, it attributes both desirable and undesirable occurrences to supernatural or magical forces, and it searches for means to win the favor of these forces.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To establish a positive connection between the members of the society&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To help society members better understand the forces controlling their food supply&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To distinguish their beliefs from those of other societies&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1217,6 +1369,11 @@
 [] The author points out problems with two popular theories.</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The author presents two theories for a historical phenomenon.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following best describes the organization of this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;A closely related theory sees theater as evolving out of dances that are primarily pantomimic, rhythmical or gymnastic, or from imitations of animal noises and sounds.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The author argues against theories expressed earlier in the passage.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The author argues for replacing older theories with a new one.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The author points out problems with two popular theories.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1239,6 +1396,11 @@
 [] Both suffer from a lack of moisture.</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Both mark forest boundaries.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following can be inferred from this passage about both the upper and lower timberlines?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In many semiarid areas there is also a lower timberline where the forest passes into steppe or desert at its lower edge, usually because of a lack of moisture.The upper timberline, like the snow line, is highest in the tropics and lowest in the Polar Regions.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Both are treeless zones.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Both are surrounded by desert areas.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Both suffer from a lack of moisture.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1261,6 +1423,11 @@
 [] resolving a dispute about the adaptability of plant seeds to bird transport</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; discussing different theories about the transport of plant seeds to Hawaii&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author of the passage is primarily concerned with&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Since the Hawaiian Islands have never been connected to other land masses, the great variety of plants in Hawaii must be a result of the long-distance dispersal of seeds, a process that requires both a method of transport and an equivalence between the ecology&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;discussing different approaches biologists have taken to testing theories about the distribution of plants in Hawaii&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;discussing the extent to which air currents are responsible for the dispersal of plant seeds to Hawaii&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;resolving a dispute about the adaptability of plant seeds to bird transport&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1283,6 +1450,11 @@
 [] silicate minerals' crystal structure</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; trace elements in the silicate minerals&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, the age of silicate minerals included in diamonds can be determined due to a feature of the&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Sometimes, however, the crystal form of the silicate inclusions is observed to resemble more closely the internal structure of diamond than that of other silicate minerals.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;trace elements in the diamond hosts&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;trace elements in the rock surrounding the diamonds&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;silicate minerals&amp;#x27; crystal structure&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1305,6 +1477,11 @@
 [x] comprise less than a third of all known types of spiders</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; comprise less than a third of all known types of spiders&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;It can be inferred from the passage that all orb-weaving spiders belong to types of spiders that&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Since most orb weavers belong either to the Araneidae or the Uloboridae families, the origin of the orb web can be determined only by ascertaining whether the families are related.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;lack venom glands&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;are included either in the Uloboridae or Araneidae families&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;share few characteristic features with other spider types&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1325,6 +1502,11 @@
 [] evidence to support Quine's claims about the problems inherent in classical empiricism
 [x] an account of Quine's counterproposal to one of the traditional assumptions of classical empiricism
 [] an overview of classical empiricism and its contributions to Quine's alternate understanding of empiricism</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; an account of Quine's counterproposal to one of the traditional assumptions of classical empiricism&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author of the passage is primarily concerned with presenting&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In classical empiricism, the truth of "All balls are red," for example, is assessed by inspecting balls; any observation of a non red ball refutes unequivocally the proposed generalization.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;criticisms of Quine's views on the proper conceptualization of empiricism&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;evidence to support Quine's claims about the problems inherent in classical empiricism&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;an overview of classical empiricism and its contributions to Quine's alternate understanding of empiricism&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1350,6 +1532,11 @@
 [x] Present findings that qualify them</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Present findings that qualify them&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The primary purpose of the passage is to treat the accepted generalizations about organ transplantation in which of the following ways?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The transplantation of organs from one individual to another normally involves two major problems: (1) organ rejection is likely unless the transplantation antigens of both individuals are nearly identical, and (2) the introduction of any unmatched transplanta&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Explicate their main features&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Suggest an alternative to them&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Examine their virtues and limitations&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Criticize the major evidence used to support them&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1372,6 +1559,11 @@
 [] Rejecting the thesis that the status of women in Mexico City during the nineteenth century actually improved</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Reviewing a historical study of the status of women in Mexico City during the nineteenth century&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The passage is primarily concerned with doing which of the following?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;According to Arrom, households headed by females and instances of women working outside the home were much more common than scholars have estimated; efforts by the Mexican government to encourage female education resulted in increased female literacy; and infl&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Analyzing the effects of economic instability on the status of women in Mexico during the nineteenth century&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Advancing a thesis explaining why women&amp;#x27;s status in Mexico City improved during the nineteenth century&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Rejecting the thesis that the status of women in Mexico City during the nineteenth century actually improved&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1394,6 +1586,11 @@
 [] animals without common ancestors sometimes evolve in similar ways</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; there are detailed skeletal similarities in the flippers of pinnipeds&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, it has been recently discovered that&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;But the recent discovery of detailed similarities in the skeletal structure of the flippers in all three groups undermines the attempt to explain away superficial resemblance as due to convergent evolution—the independent development of similarities between un&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;sea lions, seals, and walruses are all pinnipeds&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;pinnipeds are descended from animals that once lived on land&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;animals without common ancestors sometimes evolve in similar ways&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1414,6 +1611,11 @@
 [] analyzing a method of argument
 [] evaluating a point of view
 [] hypothesizing about a set of circumstances</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; summarizing the findings of an investigation&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;In the passage, the author is primarily concerned with&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;With respect to their reasons for immigrating, Cressy does not deny the frequently noted fact that some of the immigrants of the 1630&amp;#x27;s, most notably the organizers and clergy, advanced religious explanations for departure, but he finds that such explanations &lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;analyzing a method of argument&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;evaluating a point of view&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;hypothesizing about a set of circumstances&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1439,6 +1641,11 @@
 [x] skepticism</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; skepticism&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author regards the idea that traditional quantum mechanics is incomplete with&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Rather, he held that it is incomplete: in quantum mechanics the motion of a particle must be described in terms of probabilities, he argued, only because some parameters that determine the motion have not been specified.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;approval&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;surprise&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;indifference&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;apprehension&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1461,6 +1668,11 @@
 [] It evaluates an explanation and finally accepts that explanation.</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; It discusses an apparent inconsistency and suggests a reason for it.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following best describes the passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;For a brief moment in 1967, however, it appeared that the two movements might unite under the leadership of Martin Luther King, Jr.King&amp;#x27;s role in the antiwar movement appears to require little explanation, since he was the foremost advocate of nonviolence of h&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;It outlines a sequence of historical events.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It shows why a commonly held view is inaccurate.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It evaluates an explanation and finally accepts that explanation.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1483,6 +1695,11 @@
 [] criticizing experimental results</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; suggesting an answer to a theoretical question&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The passage is primarily concerned with&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Moreover, even if Earth rocks were freed by meteorite impact, Mars&amp;#x27;s orbit is much larger than Earth&amp;#x27;s, so Phinney estimates that the probability of these rocks hitting Mars is about one-tenth as great as that of Mars&amp;#x27;s rocks hitting Earth.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;presenting an argument to support a particular hypothesis&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;questioning the assumptions of a research project&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;criticizing experimental results&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1505,6 +1722,11 @@
 [] The public has continued to enjoy Twain's story, but the last part of the novel seems too violent to American minds.</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The public had too strong a belief in the doctrine of progress to accept the cynicism demonstrated at the conclusion of Twain's novel.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, which of the following is a true statement about the reception of A Connecticut Yankee in King Arthur's Court by the American public?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;None of these translations to screen and stage, however, dramatize the anarchy at the conclusion of A Connecticut Yankee, which ends with the violent overthrow of Morgan's three-year-old progressive order and his return to the nineteenth century, where he appa&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Twain's novel received little public recognition until the work was adapted for motion pictures and plays.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Although the public enjoyed Twain's humor, his use of both sixth-century and nineteenth-century characters confused many people.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The public has continued to enjoy Twain's story, but the last part of the novel seems too violent to American minds.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1527,6 +1749,11 @@
 [x] describing and cautioning</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; describing and cautioning&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;In the passage, the author is primarily concerned with&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In humans excessive intake (for adults, over 4 milligrams per day) over many years can lead to skeletal fluorosis, a well-defined skeletal disorder, and in some plant species, fluoride is more toxic than ozone, sulfur dioxide, or pesticides.Some important ques&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;analyzing and categorizing&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;comparing and contrasting&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;synthesizing and predicting&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1549,6 +1776,11 @@
 [] To suggest that contemporary American Indian writers have sacrificed traditional values for popular literary success</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To illustrate how the author believes that members of the Native American Renaissance have broadened their potential audience&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following is most likely one of the reasons that the author mentions the work of N. Scott Momaday?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The appreciation of traditional oral American Indian literature has been limited, hampered by poor translations and by the difficulty, even in the rare culturally sensitive and aesthetically satisfying translation, of completely conveying the original&amp;#x27;s verse &lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To emphasize the similarities between Momaday&amp;#x27;s writings and their European literary models&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To demonstrate the contemporary appeal of traditional Native American oral literature&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To suggest that contemporary American Indian writers have sacrificed traditional values for popular literary success&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1569,6 +1801,11 @@
 [] A pacifist state in which the individuals are strongly opposed to the use of violence or aggression to settle disputes.
 [] A democratic society in which the voice of the majority rules.
 [] A parliamentary society in which a few members, organized as a cabinet wield executive power.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; A totalitarian society in which citizens' "policing" of each other's actions helps to maintain the status quo.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The inner workings in a honeybee hive that regulate reproduction, as they are described in the passage, are most similar to which of the following types of human societies?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Typically the queen honeybee is mother to all the bees in a hive; after mating with several male drones from other colonies, she lays fertilized eggs that develop into all-female worker bees and lays unfertilized eggs that become all-male drones.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;A pacifist state in which the individuals are strongly opposed to the use of violence or aggression to settle disputes.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;A democratic society in which the voice of the majority rules.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;A parliamentary society in which a few members, organized as a cabinet wield executive power.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1594,6 +1831,11 @@
 [x] expanded the conventional view of nineteenth-century feminism</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; expanded the conventional view of nineteenth-century feminism&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author asserts that the historians discussed in the passage have&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Nineteenth-century feminists and anti-feminist alike perceived the suffragists&amp;#x27; demand for enfranchisement as the most radical element in women&amp;#x27;s protest, in part because suffragists were demanding power that was not based on the institution of the family, wom&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;influenced feminist theorists who concentrate on the family&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;honored the perceptions of the women who participated in the women suffrage movement&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;treated feminism as a social force rather than as an intellectual tradition&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;paid little attention to feminist movements&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1616,6 +1858,11 @@
 [] Animals on the periphery of a group tended to bear marks that were more distinctive to predators than animals located in the interior of the group.</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The risk of capture for individuals in a group was the same, whether they were located in the interior of the group or on its periphery.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;It can be inferred from the passage that in species in which vigilant behavior is directed at predators, the tendency of the animals to be more vigilant in smaller groups than in larger ones would most likely be minimized if which of the following were true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;If individuals on the edge of a group are more vigilant because they are at greater risk of being captured, then individuals on average would have to be more vigilant in smaller groups, because the animals on the periphery of a group form a greater proportion &lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The vigilance of animals on the periphery of a group always exceeded that of animals located in its interior, even when predators were not in the area.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Animals on the periphery of a group tended to be less capable of defending themselves from attack by predators than animals located in the interior of the group.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Animals on the periphery of a group tended to bear marks that were more distinctive to predators than animals located in the interior of the group.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1638,6 +1885,11 @@
 [x] Its results are still considered by some to be evidence for the advantages of microgravity protein crystal growth.</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Its results are still considered by some to be evidence for the advantages of microgravity protein crystal growth.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, which of the following is true about the Space Lab experiment conducted in 1983?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;That experiment is still cited as evidence that growing crystals in microgravity can increase crystal size: the authors reported that they grew lysozyme protein crystals 1,000 times larger than crystals grown in the same device on Earth.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;It was the first experiment to take place in the microgravity environment of space.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It was the first experiment in which researchers in space were able to grow lysozyme protein crystals greater in size than those grown on Earth.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Its results have been superseded by subsequent research in the field of microgravity protein crystal growth.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1660,6 +1912,11 @@
 [x] present evidence that may help to resolve an apparent contradiction</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; present evidence that may help to resolve an apparent contradiction&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The primary purpose of the passage is to&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Since one consequence of adrenaline release in an animal is an increase in blood glucose levels, we examined the effects of glucose on memory in rats.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;reconcile two opposing theories&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;compare two different explanations for a phenomenon&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;describe experimental research that appears to support an unpopular theory&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1682,6 +1939,11 @@
 [] is similar on the two sides of a rift unless a suture divides the two sides</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; cannot provide information about the nature of underlying rocks&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Part of the Harris and Gass hypothesis about the Red Sea rift would be weakened if it could be demonstrated that the composition of upper rock layers&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Geologists Harris and Gass hypothesized that the Red Sea rift developed along the line of a suture (a splice in the Earth&amp;#x27;s crust) formed during the late Proterozoic era, and that significant observable differences in the composition of the upper layers of roc&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;cannot cause a suture to develop&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;has no effect on where a suture will occur&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;is similar on the two sides of a rift unless a suture divides the two sides&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1702,6 +1964,11 @@
 [x] Describing a method of analysis that provides information regarding the relation between the carbon dioxide content of the Earth's atmosphere and global temperature
 [] Presenting information that suggests that global temperature has increased over the last 160,000 years
 [] Describing the kinds of information that can be gleaned from a careful analysis of the contents of sheets</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Describing a method of analysis that provides information regarding the relation between the carbon dioxide content of the Earth's atmosphere and global temperature&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;In the passage, the author is primarily concerned with doing which of the following?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Estimates of global temperature based on this information, combined with analysis of the carbon dioxide content of air trapped in ice deep beneath the polar surface, suggest that during periods of postglacial warming carbon dioxide in the Earth's atmosphere in&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Describing a new method of estimating decreases in global temperature that have occurred over the last 160,000 years&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Presenting information that suggests that global temperature has increased over the last 160,000 years&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Describing the kinds of information that can be gleaned from a careful analysis of the contents of sheets&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1727,6 +1994,11 @@
 [x] obscures women's contributions to literature</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; obscures women's contributions to literature&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;It can be inferred from the passage that the author views the division of literature into periods based on men's writing as an approach that&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Margaret Anne Doody, for example, suggests that during 'the period between the death of Richardson and the appearance of the novels of Scott and Austen,' which has 'been regarded as a dead period,' late-eighteenth-century women writers actually developed 'the &lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;makes distinctions among literary periods ambiguous&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;is appropriate for evaluating only premodern literature&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;was misunderstood until the advent of feminist criticism&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;provides a valuable basis from which feminist criticism has evolved&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1749,6 +2021,11 @@
 [] Frequent travel, due to limited water supplies in the Middle East, created many opportunities for trade with neighboring societies.</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Many useful and decorative raw materials cannot be found naturally in the Middle East but are available from neighboring regions.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the paragraph, why has trade been so important throughout the history of the Middle East&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Ancient demands for obsidian (a black volcanic rock useful for making mirrors and tools) led to trade with Armenia to the north, while jade for cutting tools was brought from Turkistan, and the precious stone lapis lazuli was imported from Afghanistan.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The rare and valuable metals and stones found in Middle Eastern deserts have always been in high demand in surrounding areas.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Growing conditions throughout the Middle East are generally poor, forcing Middle Eastern people to depend on imported grain.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Frequent travel, due to limited water supplies in the Middle East, created many opportunities for trade with neighboring societies.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1771,6 +2048,11 @@
 [] Elements were chemically most similar to those just before and after them in the order.</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Elements with similar chemical properties appeared in the listing at regular intervals.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this passage, what pattern did scientists notice when the known elements were written in order of increasing atomic mass?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The periodic table is a chart that reflects the periodic recurrence of chemical and physical properties of the elements when the elements are arranged in order of increasing atomic number (the number of protons in the nucleus).&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The elements of the group of alkali metals were the first elements in the order of increasing atomic mass.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Repetition of the same atomic masses for elements in different groups appeared.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Elements were chemically most similar to those just before and after them in the order.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1793,6 +2075,11 @@
 [x] Terrestrial planets travel in a different direction than Jovian planets do.</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Terrestrial planets travel in a different direction than Jovian planets do.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, each of the following statements comparing terrestrial planets with Jovian planets is true EXCEPT:&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The planets in our solar system fall into two groups: the terrestrial (Earth-like) planets (Mercury, Venus, Earth, and Mars) and the Jovian (Jupiter-like) planets (Jupiter, Saturn, Uranus, and Neptune).&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Terrestrial planets are closer to the Sun than Jovian planets.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Terrestrial planets have smaller diameters than Jovian planets.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Terrestrial planets have smaller masses than Jovian planets.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1815,6 +2102,11 @@
 [x] Commercial routes over land had become blocked because of political events.</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Commercial routes over land had become blocked because of political events.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage why was it necessary to find a new way for European merchants to reach the East?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Widely reported, if somewhat distrusted, accounts by figures like the famous traveler from Venice, Marco Polo, of the willingness of people in China to trade with Europeans and of the immensity of the wealth to be gained by such contact made the idea irresisti&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;People in China were finally ready to trade with Europeans.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The European economy was failing because there was no trade with the East.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Traditional ways of trading with the East had become very costly.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1837,6 +2129,11 @@
 [] No one has taken up serious investigation on the mystery of the Bermuda Triangle.</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The missing ships and planes around the Bermuda Triangle have aroused public curiosity.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What main point is the author trying to make?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;A few die hard rationalists believe that there is no mystery element that needs to be explained as the figures pertaining to wrecks is common when there is such exceeding traffic on sea.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The Bermuda Triangle has always been shrouded in mystery.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The missing ships in the Bermuda Triangle’s domain perhaps were lost to identifiable reasons.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;No one has taken up serious investigation on the mystery of the Bermuda Triangle.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1859,6 +2156,11 @@
 [x] Life of immoderation is neither natural nor desirable.</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Life of immoderation is neither natural nor desirable.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following most accurately summarizes the opinion of the author in the text?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In fact, the contrary is true, for as the people advance they learn to master the forces of nature and with these forces under control they are able to lead better, healthier lives; but if they become too soft and luxurious, there is decay of moral and physica&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Civilization must suffer the consequences of self-control and self-denial.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Unnecessary waste of life is the natural consequence of civilization.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;People should live in comfort and health beyond what is now considered old age.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1881,6 +2183,11 @@
 [] he changed people's ideas about businessmen</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; he introduced new sales practices&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The best description of Eaton is that&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;He offered a unique style of trade, but as was expected, all the other shopkeepers laughed at him, believing he would eventually fail.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;he was the richest merchant in Toronto&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;he was a successful technical inventor&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;he changed people&amp;#x27;s ideas about businessmen&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1903,6 +2210,11 @@
 [] all countries should bring the population growth under control.</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; rich countries exercise worse influence on environment than poor countries.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;In the author&amp;#x27;s opinion,&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;It is a very common belief that the problems of the population explosion are caused mainly by poor people living in poor countries who do not know enough to limit their reproduction.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;developing countries should be responsible for environmental problems.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;overpopulation in the world is created by the developed countries.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;all countries should bring the population growth under control.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1925,6 +2237,11 @@
 [] The Kenyan coast has over the centuries served host to diverse communities and cultures.</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Cushitic speaking people moved into today’s Kenyan territory around 2000 years ago.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following statements is not true with reference to Kenya?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The Kenyan coast served host to communities of iron workers, subsistence farmers, hunters and fishermen who supported the economy with agriculture, fishing, metal production and trade with foreign countries.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Settlers from Arab Countries constitute a significant fraction of Kenya’s population today.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Arab traders started paying regular visits to Kenya ever since the turn of the Common Era.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The Kenyan coast has over the centuries served host to diverse communities and cultures.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1947,6 +2264,11 @@
 [] to find the causes of the failure in the device.</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; to find out if there was water on Mars.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The main task of Mars Global Surveyor is&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Mars Global Surveyor is the oldest of five NASA robotic devices, which is designed to find out signs that Mars once had water; and it had been taking detailed pictures of the red planet for a decade.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;to take pictures of the red planet.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;to work out the problems of its motor.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;to find the causes of the failure in the device.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1969,6 +2291,11 @@
 [x] Sought an explanation of why certain sex ratios exist and remain stable.</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Sought an explanation of why certain sex ratios exist and remain stable.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author suggests that the work of Fisher and Hamilton was similar in that both scientists&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;By Fisher&amp;#x27;s genetic argument that the sex ratio will be favored which maximizes the number of descendants an individual will have and hence the number of gene copies transmitted, it should pay a female to produce equal numbers of sons and daughters.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Conducted their research at approximately the same time.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sought to manipulate the sex ratios of some of the animals they studied.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Studied game theory, thereby providing important groundwork for the later development of strategy theory.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1991,6 +2318,11 @@
 [x] to discuss the varying views about the start and end of World War II.</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; to discuss the varying views about the start and end of World War II.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The main purpose of the text is&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;According to AJP Taylor, two wars were fought simultaneously; the Sino-Japanese War in East Asia and a Second European War in Europe and her colonies.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;to throw light on the views of AJP Taylor about the beginning of World War II.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;to highlight the generally held view about the start and end of World War II.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;to prove that World War II did not end on particular day throughout the world.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2013,6 +2345,11 @@
 [] English is the native language of more than half a billion people of the world.</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; English has become the dominant language of international communication.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following most accurately summarizes the opinion of the author in the text?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Two thirds of the world’s science writing is in English, and English is the main language of technology, advertising, media, international airports, and air traffic controllers.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Small enclaves of English speakers have grown in various parts of the world.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Over the past 500 years, small English communities have proliferated all over the world.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;English is the native language of more than half a billion people of the world.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2035,6 +2372,11 @@
 [x] was significantly larger than the site today.</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; was significantly larger than the site today.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The ancient city of Angkor ( )&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Extending over an area of 120 sq mi (32.3 sq km), the ruins contain some of the most imposing monuments in the world, including about a thousand temples, mainly Hindu and some Buddhist; the ancient city, however, had an extent perhaps nearly 10 times that size&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;was similar in size to the Tonlé Sap lake.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;covered an area of approximately 750,000 square metres.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;was built at the ruins of a thousand temples.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2057,6 +2399,11 @@
 [] Excise taxes are levied on goods to which sales tax does not apply, while tariffs only apply to goods With sales tax imposed.</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Excise taxes are levied on goods produced and consumed in one country, while tariffs apply to imports.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this text, how do excise taxes usually differ from tariffs?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;They differ from tariffs, which usually apply only to foreign-made goods, and from sales taxes, which typically apply to all commodities other than those specifically exempted.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Excise taxes are levied on all products, while tariffs apply to government-made goods.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Excise taxes are levied on specifically identified commodities, while tariffs apply to all goods.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Excise taxes are levied on goods to which sales tax does not apply, while tariffs only apply to goods With sales tax imposed.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2079,6 +2426,11 @@
 [] Essays are opportunities for students to express their ideas.</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Essays are basically what your lecture has said throughout the course.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, which statement below is NOT true about essays?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Essays are used as an assessment tool to evaluate your ability to research a topic and construct an argument, as well as your understanding of subject content.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Essays should evaluate aspects of the course in a greater depth.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Essays should be written in formal academic style.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Essays are opportunities for students to express their ideas.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2101,6 +2453,11 @@
 [] To foresee a new academic trend.</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To introduce a new academic subject to us.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the aim of the author?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Historians have to be aware of genre, plot and rhetorical techniques in the creation both of their sources and their own arguments, while linguists need to appreciate the social and political concerns that are woven into literary works.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To distinguish the two subjects in terms of academic importance.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To criticize the combination of the two subjects.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To foresee a new academic trend.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2123,6 +2480,11 @@
 [] He completed his degree in 1910.</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; His abilities were evident at a young age.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What does the reader of this text learn about John Robertson?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The year was 1910, and those assembled were to hear not only of his generosity to the University, which enabled it to contribute to the pioneering research into tropical diseases being carried out at that time, but also of his humanitarian work in southern Afr&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;He was born in Africa.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;He studied medicine.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;He completed his degree in 1910.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2147,6 +2509,11 @@
 [] Change their understanding of numbers.</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Adding information to other data they have collected.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this passage, what do social scientists use written sources to do?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;When we want to understand their value as social science evidence we need to forget how familiar we are with first person accounts and everyday speech - for example, in newspapers, magazines, and books - and learn a different approach to them.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Formulating questionnaires and interview questions.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Advising them on how to collect qualitative evidence.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Change their understanding of numbers.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2170,6 +2537,11 @@
 [] emphasize the main argument of the essay</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; increase the length of essay&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the writer, a student might repeat himself to _____ .&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Certainly a lot of what your high school writing teachers taught you will be useful to you as you approach writing in college you will want to write clearly, to have an interesting and arguable thesis, to construct paragraphs that are coherent and focused, and&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;write a conclusion for the essay&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;remind the teacher of what he has written&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;emphasize the main argument of the essay&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2192,6 +2564,11 @@
 [] This method can be applied to all cancers.</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The virus will be delivered by blood.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, which statement below is true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Prof Seymour’s innovative solution is to mask the virus from the body’s immune system, effectively allowing the viruses to do what chemotherapy drugs do — spread through the blood and reach tumors.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;It is not a new way to fight cancer.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The experiment of this method has succeed.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;This method can be applied to all cancers.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2214,6 +2591,11 @@
 [x] Money is related to civilization.</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Money is related to civilization.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What can we infer from this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;As he became more civilized, however, he began to want better shelter, more efficient tools and weapons, and more comfortable and more lasting clothing than those that could be provided by the work of his own unskilled hands.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;A) People create money for more efficient tools and weapons.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;There is a little need of money in the earliest stage.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Previous people can make advanced tools by themselves.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2236,6 +2618,11 @@
 [] To decrease the use of melatonin.</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To introduce melatonin.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is purpose of this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Experts strongly urge people to consult their doctor or a sleep specialist before taking melatonin, in part because the supplement does not address many underlying health problems that may be disrupting sleep.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To persuade people to take melatonin.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To induce sleeping problems.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To decrease the use of melatonin.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2258,6 +2645,11 @@
 [x] They seldom used sedge root in their work.</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; They seldom used sedge root in their work.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which description about Pomo is false?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Pomo, the Native Americans of northern California, were highly skilled at basketry, using the reeds, grasses, barks, and roots they found around them.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Pomo people were good at handwork.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;They used limited materials in their work.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Their baskets have various designs.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2280,6 +2672,11 @@
 [] The advantages of televisions.</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The change of politics given by televisions.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the main idea of this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Television has transformed politics in the United States by changing the way in which information is disseminated, by altering political campaigns, and by changing citizen&amp;#x27;s patterns of response to politics.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The political patterns in America.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The change of audience in speeches.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The advantages of televisions.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2302,6 +2699,11 @@
 [x] A definite thesis is necessary for explicatory essay.</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; A definite thesis is necessary for explicatory essay.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, which statement below is true about explicatory essay?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;An explication, or “explicatory” essay is used to explain and interpret a piece of literature such as a poem, a play, a novel, or a short story.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Explicatory essay aims to analyze a piece of poem.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Authors of literary works write explicatory essay.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Explicatory essay focuses on examining only short literary works.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2324,6 +2726,11 @@
 [] People now can enjoy the work on screen, TV and stage.</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The famous work of Ernest Hemingway-A Farewell to Arms-describes the Italian campaign after the First World War.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, which statement below is NOT true about A Farewell to Arms?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Written in the first-person point of view, the story shows Frederic Henry, a lieutenant working as an ambulance driver in the Italian forces is involved in a love affair with a nurse, Catherine Barkley.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;As one of the best literary works of Ernest Hemingway, A Farewell to Arms was published in the late 1920s.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;In addition to the love story, Hemingway also mentions about how absurd war is and how he loses his love.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;People now can enjoy the work on screen, TV and stage.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2346,6 +2753,11 @@
 [] Arthur Miller’s family enjoyed a prosperous life even during the Depression.</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; People around the world who were interested in this play were able to enjoy it after it became successful.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, which of the following can be inferred?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The story of the play revolves around an unfortunate middle-class man who ruins his life, chasing the idea of the American Dream.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Produced in the late 1940s, the play did not achieve great success immediately.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The author of the play, Arthur Miller, did not receive the Pulitzer Prize in his lifetime.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Arthur Miller’s family enjoyed a prosperous life even during the Depression.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2368,6 +2780,11 @@
 [] To be healthy, people should avoid eating foods that are processed and provide less nutrients.</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To make sure that you get enough nutrients, you should focus on eating a few specific kinds of foods.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, which statement below is NOT true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Many people realize that healthy eating habits can help support a healthy weight, manage or improve chronic diseases and maintain overall good health.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Maintaining healthy eating habits is conducive to the management or even the improvement of chronic diseases.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It is said in the text that small changes over a longer period can help to develop healthy eating habits.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To be healthy, people should avoid eating foods that are processed and provide less nutrients.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2390,6 +2807,11 @@
 [] develop more quickly than at present.</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; slow down the rate of its development.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The Norwegian Government would prefer the oil industry to __ .&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;A new law limits exploration to an area south of the southern end of the long coastline; production limits have been laid down (though these have already been raised); and oil companies have not been allowed to employ more than a limited number of foreign work&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;provide more jobs for foreign workers.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;sell the oil it is producing abroad.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;develop more quickly than at present.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2412,6 +2834,11 @@
 [] To ban the advertisement along the highway.</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Giving some suggestions to make stricter driving law.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the main idea of this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The driving test should be standardized and made far more difficult than it is; all the drivers should be made to take a test every three years or so; the age at which young people are allowed to drive any vehicle should be raised to at least 21; all vehicles &lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The lax driving law in some countries.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The driving test should be standardized.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To ban the advertisement along the highway.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2434,6 +2861,11 @@
 [x] To create better networks of public transportation.</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To create better networks of public transportation.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which one is not related to mass transportation according to this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;By opening vast areas of unoccupied land for residential expansion, the omnibuses, horse railways, commuter trains, and electric trolleys pulled settled regions outward two to four times more distant from city centers than they were in the premodern era.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The increasing of available land of a city.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To expand the urban area.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To make urban life unstable.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2456,6 +2888,11 @@
 [] To make more money for advertiser.</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To give information.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is another use of advertisement except selling goods?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Their critics seem to resent them because they have a flair for self-promotion and they have so much money to throw around.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To propagate.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To increase people’s reading ability.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To make more money for advertiser.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2478,6 +2915,11 @@
 [] To provide solutions for climate change.</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To call for the action to combat global warming.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the author’s main purpose to write this passage?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The planet is already seeing the effects of global warming: Arctic sea ice is declining, sea levels are rising, wildfires are becoming more severe and animal migration patterns are shifting.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To state the fact of climate change.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To state the fact of global warming.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To provide solutions for climate change.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2498,6 +2940,11 @@
 [] Baking powder is different from baking soda in that the former combines the latter with two acids.
 [] Upon contacting with yogurt, baking soda immediately releases carbon dioxide bubbles, causing the baked goods to change.
 [] Temperature and moisture are necessary for the sodium aluminum sulfate to react with the sodium bicarbonate.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Unlike baking soda which extends the leavening process, baking powder can accelerate the process.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, which of the following statement is NOT true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;On the other hand, baking powder is a combination of baking soda (sodium bicarbonate) and two acids, often monocalcium phosphate and sodium aluminum sulfate.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Baking powder is different from baking soda in that the former combines the latter with two acids.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Upon contacting with yogurt, baking soda immediately releases carbon dioxide bubbles, causing the baked goods to change.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Temperature and moisture are necessary for the sodium aluminum sulfate to react with the sodium bicarbonate.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2523,6 +2970,11 @@
 [] DIT helps us with weight gain.</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; DIT has negative correlation with weight gain.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following statements is true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Typically, the chewing process reportedly enhances the energy expenditure associated with the metabolism of food and increases intestinal motility — all summing up to an increased heat generation in the body after food intake, known as diet-induced thermogenes&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The relation between weight loss and slow eating and thorough chewing is not clear.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Slow eating doesn’t help prevent obesity.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Slow eating will ease the intestinal motility.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DIT helps us with weight gain.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2545,6 +2997,11 @@
 [] encourage people to protect microorganisms.</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; introduce two kinds of microorganisms responsible for fermentation.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The purpose of the text is to ____ .&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;A biologist would probably say fermentation is the anaerobic production of energy, meaning that microorganisms that don&amp;#x27;t need oxygen to accomplish metabolization to fuel their bodies transform nutrients into energy in the absence of oxygen.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;explain the origins and meanings of the word “ferment”.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;demonstrate two different types of fermentation.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;encourage people to protect microorganisms.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2567,6 +3024,11 @@
 [x] is not as acute as once thought by farmers.</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; is not as acute as once thought by farmers.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, foodborne risk from birds ___.&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Birds like starlings that flock in large numbers and forage on the ground near cattle are more likely to spread pathogenic bacteria to crops like lettuce, spinach and broccoli, according to the study of food safety risk and bird pathogens.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;should be emphasized greatly.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;will cause many diseases.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;will increase in the future.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2589,6 +3051,11 @@
 [] The Quaker oats usually take some time to become edible.</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Steel-cut oats differ from Scottish oats in their different ways of production.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, which of the following statement is true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;As a result, steel-cut oats cook in about half the time of whole oat groats but still have that same chewy, subtle nutty flavor and may also be a bit creamier.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Steel-cut oats taste differently than whole oat groats because of the additional procession.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The classic rolled oats are flat and oval before they have been steamed, rolled and pressed.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The Quaker oats usually take some time to become edible.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2611,6 +3078,11 @@
 [] It has dozens of unique gene families compared to other conifers.</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; It has genes that are beneficial to recovery.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, which statement is true about coast red wood?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Scientists have completed the sequences for the coast redwood, which helps to better explain the genetic basis for these species’ ability to adapt to their changing environments.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Its genome evolved from multiple species.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Coast red wood sequencing is a simple task for scientists.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It has dozens of unique gene families compared to other conifers.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2633,6 +3105,11 @@
 [] To install a wireless adapter on your PC.</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; To uninstall the wireless adapter on your computer.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;When your PC cannot connect to a wireless network, which of the following cannot help you to address the problem?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;If you want to take advantage of public WiFi hot spots or your own home-based network, the first thing you&amp;#x27;ll need to do is make sure your computer has the right gear.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;To check whether there are WiFi hot spots available around.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To check whether your computer has a wireless transmitter.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;To install a wireless adapter on your PC.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2655,6 +3132,11 @@
 [] have lower and lower effect if bees repeatedly expose to them.</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; reduce bees’ fertility rates.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;From the study, pesticides ___&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;New study from researchers at the University of California, Davis, finds that pesticides not only directly affect bee health, but effects from past exposure can carry over to future generations.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;indirectly have an influence on bees.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;promote population growth of bees.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;have lower and lower effect if bees repeatedly expose to them.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2677,6 +3159,11 @@
 [] will not be heard by dogs</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; with high-frequency and intermittence make dogs uneasier&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the study, noises ___.&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;It’s well established that sudden loud noises, such as fireworks or thunderstorms, commonly trigger a dog’s anxiety, a new study finds even common noises, such as a vacuum or microwave, can be a trigger.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;make dogs happier&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;with low-frequency and continuousness make dogs more anxious&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;will not be heard by dogs&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2699,6 +3186,11 @@
 [] There are different routes for the transmission of data in a packet-switching network.</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The receiving computer can determine whether or not the package is intact all by itself.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, which description below of the transmission process is NOT true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Each of these packages gets a wrapper that includes information on the sender&amp;#x27;s address, the receiver&amp;#x27;s address, the package&amp;#x27;s place in the entire message, and how the receiving computer can be sure that the package arrived intact.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;In a packet-switching network, the data cannot be transmitted without being cut into packages.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Apart from the data, a package also carries with it some other information.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;There are different routes for the transmission of data in a packet-switching network.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2721,6 +3213,11 @@
 [] 100%</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; 50%&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;How much irrigation water is the most beneficial in maintaining the grape’s flavor profile and yield according to the research?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;California grape growers in coastal areas can use less water during times of drought and cut irrigation levels without affecting crop yields or quality, according to a new study out of the University of California, Davis.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;25%&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;30%&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;100%&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2743,6 +3240,11 @@
 [] comparing opinions from different sides.</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; presenting conclusion and supporting evidence.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The author develops the passage mainly by ___ .&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;In an ongoing longitudinal study, researchers tested the saliva of 229 17-year-olds, many of whom had lived at or below the poverty level between the ages 10 and 16, for their levels of cortisol — a hormone in the blood.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;providing typical examples.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;following natural time order.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;comparing opinions from different sides.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2765,6 +3267,11 @@
 [x] Cotton price will decrease with the spread of Fusarium wilt disease.</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Cotton price will decrease with the spread of Fusarium wilt disease.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which statement below is not true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;And this can be a very damaging disease in terms of greatly reducing yields, and to some extent, even making cotton uneconomical as a crop in a region.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Pima cotton is often used for fine clothes.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Fusarium wilt disease will bring serious damage to cotton.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Cotton price will increase with the spread of Fusarium wilt disease.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2788,6 +3295,11 @@
 [] is useless for improving the status of stray animals</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; supports that treatable animals should not be euthanized&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, Animal Shelter Assistance Program ___ .&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The funding reflects the governor’s commitment to providing resources that can help communities realize the state’s long-held policy that “no adoptable or treatable animal should be euthanized.” The Shelter set up a grant process, create and distribute educati&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;hasn&amp;#x27;t been signed yet&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;provides $45 billion for animals&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;is useless for improving the status of stray animals&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2808,6 +3320,11 @@
 [] A dictionary
 [x] A travel book.
 [] An encyclopedia.</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; A travel book.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Where does this passage most likely to appear?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Man has left his mark here too, carving out more than 110 rock tombs, many with ornate details: steps symbolising the way to heaven above the entrance, shelf cornicing and perhaps the head of Medusa to warn against tomb raiders.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;A textbook.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;A dictionary&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;An encyclopedia.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2833,6 +3350,11 @@
 [] Mr. Clark will be under arrest.</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Mr. Clark will give these antiquities to the police.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;We can infer from this passage that __&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Clark said, “My doing might inspire other people to do the same, but I’m not sure — it’s hard for people to give up something they paid for, but for me, why would you want to own something that was stolen?”&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Mr. Clark will not collect antiquities any more.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mr. Clark donates these collections to charity.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mr. Clark stole these antiquities in Asia.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Mr. Clark will be under arrest.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2855,6 +3377,11 @@
 [] You will feel calm in the Tree of Life.</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; All the buildings in this villa complex have harsh edges.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this passage, which one below is false?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;To fit with the peaceful atmosphere of the surroundings, the villas are designed with organic forms, lacking harsh edges with the exception of their angled roofs.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Tree of Life is an ideal place for stressful people.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;There are trees around the villa complex.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;You will feel calm in the Tree of Life.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2877,6 +3404,11 @@
 [] DMV needs 15 seconds to start the engine.</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; People think DMV is pragmatic.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this passage, we can know that __&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;It runs with normal rubber tires on the road, but when it needs to switch to train mode, a pair of metal wheels drop down from the vehicle’s underbelly.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;People like DMV’s appearance.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DMV can work as a plane.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;DMV needs 15 seconds to start the engine.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2899,6 +3431,11 @@
 [] can’t navigate and find food at the same time.</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; can do more processing than a supercomputer.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to this passage, we can know that fruit flies __&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Scientists at Johns Hopkins Medicine meticulously counted brain cells in fruit flies and three species of mosquitos, revealing a number that would surprise many people outside the science world.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;have about 12 billion neurons and cells in the brain.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;have more brain cells than rodents.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;can’t navigate and find food at the same time.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2921,6 +3458,11 @@
 [] When there is a fight between two families, a “Commission” will decide how to settle it.</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Families may fight with each other or work together depending on the circumstances.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;From the author’s description of Mafia, which of the following statement is true?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;At other times, they have cooperated in the interest of greater profits, sometimes even serving on a &amp;quot;Commission&amp;quot; that made major decisions affecting all the families .&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The Mafia is just a single gang that is divided into several different families.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Organized crime is believed to be related to the Mafia.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;When there is a fight between two families, a “Commission” will decide how to settle it.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2943,6 +3485,11 @@
 [] argue how easy it is to live a different lifestyle.</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; encourage people to live a healthy lifestyle.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The main purpose of the author is to ___&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;By supporting your body and mind, making some simple tweaks to your routine, and setting small goals for yourself, you can be on the path toward living a healthier, happier life.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;demonstrate how difficult it is to be healthy.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;show the disadvantages of changing lifestyles.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;argue how easy it is to live a different lifestyle.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2965,6 +3512,11 @@
 [] different ways to build up your stamina over a long period.</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; methods to improve your stamina quickly.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the passage, what might the “tricks” mentioned in the last sentence refer to?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;If you&amp;#x27;ve been relatively sedentary, you might find that you can&amp;#x27;t walk very far at first without getting sore or out-of-breath.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;suggestions on how to keep fit.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;benefits of different styles of walking.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;different ways to build up your stamina over a long period.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2987,6 +3539,11 @@
 [] Apart from making small changes to our life, controlling our genes can also make us healthier.</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; A healthier life requires various small changes to diverse aspects of our life, such as diet, exercise and so on.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;What is the main idea of the text?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Since you cannot control your genes, making changes to items you have control over can help lead to a healthier lifestyle.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Healthier lifestyles can bring people a great deal of benefits, including losing weight, being more active and feeling healthier.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Some delicate adjustments in a limited scope of areas are believed to help us to lead a healthier lifestyle.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Apart from making small changes to our life, controlling our genes can also make us healthier.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3009,6 +3566,11 @@
 [] The latest news about COVID-19 cases worldwide.</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; A more simplified and interesting description about social distancing.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;The passage is an excerpt from a longer essay. According to the last sentence, what may the remaining part of the essay be about?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The specific distance is determined by health experts and national governments, and social distancing is a recommended medical practice to help “flatten the curve,” or lower the number of COVID-19 cases throughout the world.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;More detailed professional information on the mechanisms of social distancing.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Experimental evidence about the effectiveness of social distancing.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The latest news about COVID-19 cases worldwide.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -3033,6 +3595,11 @@
 [] South Pacific</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Antarctica&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Where did the largest piece off from B-15 eventually go?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;After it started breaking up, the largest of its pieces, B-15a, drifted along the coast of Antarctica, lingered on a shallow seamount, and collided with an ice tongue, before running aground and breaking again.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Seafloor&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Chile&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;South Pacific&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -3055,6 +3622,11 @@
 [] NASA's rover, Curiosity, has had recent software upgrades that have let it explore new areas of Mars looking for evidence of life.</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; Over the last four years, NASA's rover, Curiosity, has collected samples and taken photographs of Mars’ surface which have revealed evidence of water but has not confirmed evidence of life.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Choose the correct sentence that best summarizes the text.&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;While the rover has yet to confirm whether Mars once hosted living things, it has found evidence of an ancient freshwater lake in the sediments of Yellowknife Bay, the lowest point of the crater, offering tantalizing insight into the planet’s past habitability&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;NASA's rover, Curiosity, has not had recent software upgrades that have let it explore new areas of Mars looking for evidence of life.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Photographs of Mars' surface have not revealed evidence of water but have confirmed evidence of life.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;NASA's rover, Curiosity, has had recent software upgrades that have let it explore new areas of Mars looking for evidence of life.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -3077,6 +3649,11 @@
 [x] The author believes that the maps are works of art that give information about London’s destruction in World War II.</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; The author believes that the maps are works of art that give information about London’s destruction in World War II.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;Which of the following most accurately summarizes the opinion of the author in the text?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;The extent of the damage to each and every one of these buildings was logged and mapped in near real-time by surveyors, architects, engineers, and construction workers.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The author believes that the maps are a beautiful and accurate representation of pre-war London.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The author believes that the maps are an accurate representation of post-war London.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The author believes that the maps are a valuable piece of World War II history.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -3099,6 +3676,11 @@
 [] Controlling their actions, CPG receives a simple signal from the brain to switch between different modes.</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Correct answer:&lt;/strong&gt; They do not know what to do with their very sharp brains.&lt;/p&gt;&lt;p&gt;This option is correct for the question &lt;strong&gt;According to the text, what is the reason teens can be so clever, accomplished and responsible and reckless at the same time in terms of brain activities?&lt;/strong&gt; because it is the only choice that stays aligned with the passage. The key evidence is: &lt;em&gt;Easily, according to two physicians at Children&amp;#x27;s Hospital Boston and Harvard Medical School( HMS) who have been exploring the unique structure and chemistry of the adolescent brain.&lt;/em&gt; This supports the idea in the correct answer without adding a new claim or shifting the meaning.&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Why the other options are incorrect:&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Their brains are the same as adults&amp;#x27; but with fewer miles on it.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Their brains are so small that they cannot deal with so much information.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Controlling their actions, CPG receives a simple signal from the brain to switch between different modes.&lt;/strong&gt; is incorrect because the passage does not support it as the answer to this question. It changes the focus, cause, scope, or detail that the passage actually gives.&lt;/li&gt;&lt;/ul&gt;</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(release): Release V2.0.11 — CRM access check latency fix, security hardening, performance upgrade, and Read Aloud workspace redesign
</commit_message>
<xml_diff>
--- a/public/database/RMCSA/RMCSA/RMCSA.xlsx
+++ b/public/database/RMCSA/RMCSA/RMCSA.xlsx
@@ -487,8 +487,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that analyzing reading passages requires you to be extremely precise—you must only use the information given in the text. Let's break down this passage and question together. You did a great job identifying the correct answer, and now we will solidify your understanding of why the others are incorrect!&lt;/p&gt;
-&lt;h3&gt;✅ Analysis of the Correct Answer&lt;/h3&gt;
+          <t>&lt;h3&gt;✅ Analysis of the Correct Answer&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;Cathedral staff were reluctant to act too quickly.&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Why this is correct:&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
@@ -539,8 +538,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that mastering the "Main Purpose" question is all about reading between the lines and identifying the author's core message. Don't get distracted by the details; focus on the big picture! Let's break down this passage together.&lt;/p&gt;
-&lt;h3&gt;🎯 Analysis of the Correct Answer&lt;/h3&gt;
+          <t>&lt;h3&gt;🎯 Analysis of the Correct Answer&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;to highlight the potential benefits of geothermal power for Britain&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Why this is correct:&lt;/strong&gt;&lt;/p&gt;
 &lt;ul&gt;
@@ -592,8 +590,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello! As your PTE Academic tutor, I can tell you that analyzing the main point of a passage requires you to look beyond the surface details and identify the author's central argument. This passage is excellent because it challenges a common misconception, which is exactly what PTE questions often test!&lt;/p&gt;
-&lt;p&gt;Let's break down the passage, the question, and each option to ensure you understand the logic behind the correct answer.&lt;/p&gt;
+          <t>&lt;p&gt;Let's break down the passage, the question, and each option to ensure you understand the logic behind the correct answer.&lt;/p&gt;
 &lt;h3&gt;✅ Analysis of the Correct Answer&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;New products are not always based on new ideas.&lt;/strong&gt;&lt;/p&gt;
 &lt;h3&gt;Why this is correct:&lt;/h3&gt;
@@ -641,8 +638,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;p&gt;As an expert PTE Academic tutor, I will provide a detailed, option-level explanation to help you understand how to select the correct answer based on the passage's evidence.&lt;/p&gt;
-&lt;h3&gt;&lt;strong&gt;✅ Correct Answer Explanation&lt;/strong&gt;&lt;/h3&gt;
+          <t>&lt;h3&gt;&lt;strong&gt;✅ Correct Answer Explanation&lt;/strong&gt;&lt;/h3&gt;
 &lt;p&gt;The correct option is: &lt;strong&gt;Sea snails are being carried by submarines to places where they harm other species.&lt;/strong&gt;&lt;/p&gt;
 &lt;p&gt;&lt;strong&gt;Support:&lt;/strong&gt; This option accurately summarizes the core problem described in the passage. The text states that the limpets "latch on to the submarines... potentially spreading disease in pristine ecosystems." This directly supports the idea that the snails are being transported (carried by submarines) to new locations where they pose a threat (harm other species/ecosystems).&lt;/p&gt;
 &lt;h3&gt;&lt;strong&gt;❌ Incorrect Options Analysis&lt;/strong&gt;&lt;/h3&gt;

</xml_diff>